<commit_message>
chore: run 2026-03-15 19:31 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_15_03_2026.xlsx
+++ b/logs/Consolidado_15_03_2026.xlsx
@@ -638,10 +638,10 @@
         <v>151</v>
       </c>
       <c r="C2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -695,10 +695,10 @@
         <v>71</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -714,10 +714,10 @@
         <v>47</v>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -1958,40 +1958,40 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>15/03/2026</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>Cleanance Comedomed Peeling Cleansing Gel
 Gel de Limpeza esfoliante pele com Acne
 400 ml</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/cleanance-comedomed-peeling-cleansing-gel-8660052.html</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr"/>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr"/>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>8660052</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="H30" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -14862,12 +14862,12 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>6759973</t>
+          <t>7630905</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>
@@ -14915,40 +14915,40 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>15/03/2026</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Forticea Strengthening Revitalizing Shampoo
 Champô Fortificante Todos Tipos de Cabelo
 500 ml</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/forticea-strengthening-revitalizing-shampoo-8602496.html</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr"/>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>8602496</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -17771,43 +17771,43 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>15/03/2026</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>7434584</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -24795,38 +24795,38 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>7434584</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>
@@ -27933,12 +27933,12 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>6759973</t>
+          <t>7630905</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">

</xml_diff>